<commit_message>
Revision round: hide unreviewed status, housing gender split, drop جاهزية rubric items
- Remove all client-visible "غير مُراجَع" indicators (program banner, per-item
  pills, nav ⚠, legend pill, xlsx export warning row, Excel banner/fill).
  Keep unreviewed:true as a silent internal data flag that renders nothing.
- Housing (p2): replace region/city + eligibility-category breakdown with a
  gender split — عدد المستفيدين (ذكور) / عدد المستفيدات (إناث) per year.
- Remove firm-scored جاهزية readiness rubric items: p1_i04, p6_i04, p7_i04.
  Document-attach item p1_i05 (نماذج الحقائب) preserved.
- Regenerate al-ahli-sijillat-template.xlsx to match.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/al-ahli-sijillat-template.xlsx
+++ b/al-ahli-sijillat-template.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,14 +53,8 @@
       <color rgb="001C241F"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="006B4EA8"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -70,11 +64,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F3EFE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ECE4F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,13 +107,6 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -492,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -702,12 +684,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>نسبة جاهزية الحقيبة التدريبية (%)</t>
+          <t>نماذج الحقائب التدريبية المعتمدة</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>مصفوفة سنوات</t>
+          <t>وثيقة مرفقة</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -717,7 +699,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>الجمعية — تُقيَّم بروبريك من قرارات</t>
+          <t>الجمعية</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
@@ -736,17 +718,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>نماذج الحقائب التدريبية المعتمدة</t>
+          <t>عدد الجهات المنفذة الفعّالة (لكل سنة)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>وثيقة مرفقة</t>
+          <t>مصفوفة سنوات</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>يحتاج جلب</t>
+          <t>متوفر الآن ✓</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -770,7 +752,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>عدد الجهات المنفذة الفعّالة (لكل سنة)</t>
+          <t>التغطية الجغرافية للجهات المنفذة (عدد المدن لكل سنة)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -799,12 +781,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>مدخلات</t>
+          <t>أنشطة</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>التغطية الجغرافية للجهات المنفذة (عدد المدن لكل سنة)</t>
+          <t>عدد المبادرات التسويقية</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -838,7 +820,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>عدد المبادرات التسويقية</t>
+          <t>عدد المتاجر الإلكترونية المفتوحة (سلة)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -853,7 +835,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>الجمعية</t>
+          <t>الجمعية / سلة</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -872,7 +854,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>عدد المتاجر الإلكترونية المفتوحة (سلة)</t>
+          <t>عدد الدورات المنفذة سنوياً</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -887,7 +869,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>الجمعية / سلة</t>
+          <t>الجمعية</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr"/>
@@ -906,7 +888,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>عدد الدورات المنفذة سنوياً</t>
+          <t>عدد ساعات التدريب الإجمالية</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -940,7 +922,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>عدد ساعات التدريب الإجمالية</t>
+          <t>نسبة إكمال الدورة (Retention) (%)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -974,7 +956,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>نسبة إكمال الدورة (Retention) (%)</t>
+          <t>رضا المستفيدات عن التدريب (النتيجة سنوياً)</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1008,12 +990,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>رضا المستفيدات عن التدريب (النتيجة سنوياً)</t>
+          <t>نموذج استبيان الرضا (الكوسينير) بعد الدورة</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>مصفوفة سنوات</t>
+          <t>وثيقة مرفقة</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1042,17 +1024,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>نموذج استبيان الرضا (الكوسينير) بعد الدورة</t>
+          <t>عدد طلبات الالتحاق المستلمة</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>وثيقة مرفقة</t>
+          <t>مصفوفة سنوات</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>متوفر الآن ✓</t>
+          <t>يحتاج جلب</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1076,7 +1058,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>عدد طلبات الالتحاق المستلمة</t>
+          <t>عدد المقبولات (لكل سنة)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -1110,7 +1092,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>عدد المقبولات (لكل سنة)</t>
+          <t>عدد المستفيدات من الفئات الأولى بالرعاية (لكل سنة)</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -1120,7 +1102,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>يحتاج جلب</t>
+          <t>متوفر الآن ✓</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1139,12 +1121,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>أنشطة</t>
+          <t>مخرجات</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>عدد المستفيدات من الفئات الأولى بالرعاية (لكل سنة)</t>
+          <t>عدد المتخرجات (لكل سنة)</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1173,12 +1155,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>مخرجات</t>
+          <t>نتائج</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>عدد المتخرجات (لكل سنة)</t>
+          <t>عدد المستفيدات اللاتي أنتجن منتجاً قابلاً للبيع (لكل سنة)</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -1207,12 +1189,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>نتائج</t>
+          <t>أثر</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>عدد المستفيدات اللاتي أنتجن منتجاً قابلاً للبيع (لكل سنة)</t>
+          <t>متوسط المبيعات الشهرية عبر (سلة)</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1227,7 +1209,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>الجمعية</t>
+          <t>الجمعية / سلة</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr"/>
@@ -1246,7 +1228,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>متوسط المبيعات الشهرية عبر (سلة)</t>
+          <t>عدد الحرف التراثية المُدرَّسة (لكل سنة)</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -1261,7 +1243,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>الجمعية / سلة</t>
+          <t>الجمعية</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -1280,17 +1262,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>عدد الحرف التراثية المُدرَّسة (لكل سنة)</t>
+          <t>قائمة المتدربات (اسم + جوال + بريد + مدينة + جنس)</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>مصفوفة سنوات</t>
+          <t>قائمة مستفيدين (PII)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>متوفر الآن ✓</t>
+          <t>يحتاج جلب</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1314,7 +1296,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>قائمة المتدربات (اسم + جوال + بريد + مدينة + جنس)</t>
+          <t>قائمة المدربات (اسم + بيانات)</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -1329,7 +1311,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>الجمعية</t>
+          <t>الجمعية / هيئة التراث</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -1339,40 +1321,6 @@
       <c r="J27" s="6" t="inlineStr"/>
       <c r="K27" s="6" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>أثر</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>قائمة المدربات (اسم + بيانات)</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>قائمة مستفيدين (PII)</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>يحتاج جلب</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>الجمعية / هيئة التراث</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
-      <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="6" t="inlineStr"/>
-      <c r="I28" s="6" t="inlineStr"/>
-      <c r="J28" s="6" t="inlineStr"/>
-      <c r="K28" s="6" t="inlineStr"/>
-      <c r="L28" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1697,7 +1645,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>عدد الأسر المستفيدة حسب المنطقة/المدينة (لكل سنة)</t>
+          <t>عدد المستفيدين (ذكور) (لكل سنة)</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1731,7 +1679,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>عدد الأسر المستفيدة حسب فئة الاستحقاق التنموي (لكل سنة)</t>
+          <t>عدد المستفيدات (إناث) (لكل سنة)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -3812,7 +3760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3844,103 +3792,130 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع مع العميل — مبني من المنهجية (ن3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع في الاجتماع — بُني حرفياً من جدول ن3. تُؤكَّد الصياغة والتوافر والسنوات مع العميل. السنوات مفترَضة 2022–2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>السنوات مفترَضة 2022–2025 (تُؤكَّد مع المالك).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>المرحلة</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>البند / المؤشر</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>شكل البيان</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>الحالة (التوافر)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>المصدر / المالك</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>حالة المستند/القائمة</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>العدد</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>ملاحظات</t>
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>مدخلات</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>عدد الموظفين في الفروع</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>الجمعية / البنك</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+    </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>مدخلات</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>عدد الموظفين في الفروع</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>عدد الموظفات ذوات الدخل المستقل (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -3954,29 +3929,29 @@
       <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>مدخلات</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>عدد الموظفات ذوات الدخل المستقل (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>الجمعية / البنك</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>عدد الفروع المخصصة للبرنامج</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>البنك</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr"/>
@@ -3988,27 +3963,27 @@
       <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>مدخلات</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>عدد الفروع المخصصة للبرنامج</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>الميزانية المخصصة</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>البنك</t>
         </is>
@@ -4022,29 +3997,29 @@
       <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>مدخلات</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>الميزانية المخصصة</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>البنك</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>أنشطة</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>عدد القروض التي تم تقديمها</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>الجمعية / البنك</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr"/>
@@ -4056,27 +4031,27 @@
       <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>عدد القروض التي تم تقديمها</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>عدد القروض المقبولة (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -4090,27 +4065,27 @@
       <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>عدد القروض المقبولة (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>عدد طلبات التقديم على القروض</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -4124,27 +4099,27 @@
       <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>عدد طلبات التقديم على القروض</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>قيمة القروض المحصَّلة (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -4158,27 +4133,27 @@
       <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>أنشطة</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>قيمة القروض المحصَّلة (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>مخرجات</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>قيمة القروض المقدمة سنوياً</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -4192,27 +4167,27 @@
       <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>مخرجات</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>قيمة القروض المقدمة سنوياً</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>عدد المستفيدات الحاصلات على قروض</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>الجمعية / البنك</t>
         </is>
@@ -4226,29 +4201,29 @@
       <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>مخرجات</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>عدد المستفيدات الحاصلات على قروض</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>الجمعية / البنك</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>نتائج</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>عدد المشاريع التجارية التي تم إطلاقها</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>المستفيدات (سجل الجمعية إن وُجد)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr"/>
@@ -4258,40 +4233,6 @@
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="6" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>نتائج</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>عدد المشاريع التجارية التي تم إطلاقها</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>المستفيدات (سجل الجمعية إن وُجد)</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4304,7 +4245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4336,103 +4277,130 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع مع العميل — مبني من المنهجية (ن3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع في الاجتماع — بُني حرفياً من جدول ن3. الشريك المذكور: أروقة (احتضان). تُؤكَّد الصياغة والتوافر والسنوات. السنوات مفترَضة 2022–2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>الشريك المذكور: أروقة (احتضان). السنوات مفترَضة 2022–2025 (تُؤكَّد مع المالك).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>المرحلة</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>البند / المؤشر</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>شكل البيان</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>الحالة (التوافر)</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>المصدر / المالك</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>حالة المستند/القائمة</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>العدد</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>ملاحظات</t>
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>مدخلات</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>الميزانية السنوية المخصصة</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>البنك</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
+    </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>مدخلات</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>الميزانية السنوية المخصصة</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>المبلغ المصروف من الميزانية (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>البنك</t>
         </is>
@@ -4446,29 +4414,29 @@
       <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>مدخلات</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>المبلغ المصروف من الميزانية (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>البنك</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>حالة اتفاقيات الشراكة الفعّالة</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>حالة (اختيار)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>البنك / أروقة</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr"/>
@@ -4480,27 +4448,27 @@
       <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>مدخلات</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>حالة اتفاقيات الشراكة الفعّالة</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>حالة (اختيار)</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>أنشطة</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي التمويل المقدم للشركات الناشئة</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4514,29 +4482,29 @@
       <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>مدخلات</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>جاهزية نظام التشغيل (الحاضنة الخاصة بالبنك)</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>البنك</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>أنشطة</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>عدد ساعات التدريب (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>البنك / أروقة</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr"/>
@@ -4548,27 +4516,27 @@
       <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>إجمالي التمويل المقدم للشركات الناشئة</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>عدد جلسات الإرشاد الفردية (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4582,27 +4550,27 @@
       <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>عدد ساعات التدريب (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>عدد طلبات الالتحاق (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4616,27 +4584,27 @@
       <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>عدد جلسات الإرشاد الفردية (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>عدد المقبولين (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4650,27 +4618,27 @@
       <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>عدد طلبات الالتحاق (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>عدد فعاليات الربط (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4684,27 +4652,27 @@
       <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>أنشطة</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>عدد المقبولين (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>عدد المستثمرين المشاركين (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4718,27 +4686,27 @@
       <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>أنشطة</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>عدد فعاليات الربط (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>مخرجات</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>عدد الاتفاقيات الاستثمارية الموقعة (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4752,27 +4720,27 @@
       <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>أنشطة</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>عدد المستثمرين المشاركين (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>مخرجات</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي قيمة الاتفاقيات الاستثمارية (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4786,27 +4754,27 @@
       <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>مخرجات</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>عدد الاتفاقيات الاستثمارية الموقعة (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>عدد رواد الأعمال المحتضنين (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4820,27 +4788,27 @@
       <c r="L18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>مخرجات</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>إجمالي قيمة الاتفاقيات الاستثمارية (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>عدد الشركات المحتضنة (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4854,27 +4822,27 @@
       <c r="L19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>مخرجات</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>عدد رواد الأعمال المحتضنين (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>نتائج</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>عدد الشركات الباقية بعد سنتين (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4888,27 +4856,27 @@
       <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>مخرجات</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>عدد الشركات المحتضنة (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>نتائج</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>عدد الشركات الباقية بعد 5 سنوات (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4922,27 +4890,27 @@
       <c r="L21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>نتائج</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>عدد الشركات الباقية بعد سنتين (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>عدد الشركات المحققة لإيرادات (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4956,27 +4924,27 @@
       <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>نتائج</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>عدد الشركات الباقية بعد 5 سنوات (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي الوظائف المولَّدة (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -4990,27 +4958,27 @@
       <c r="L23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>نتائج</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>عدد الشركات المحققة لإيرادات (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>عدد الوظائف للسعوديين (لكل سنة)</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -5024,27 +4992,27 @@
       <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>نتائج</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>إجمالي الوظائف المولَّدة (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>أثر</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>إجمالي إيرادات الشركات المتخرجة</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>مصفوفة سنوات</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج جلب</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>البنك / أروقة</t>
         </is>
@@ -5056,74 +5024,6 @@
       <c r="J25" s="6" t="inlineStr"/>
       <c r="K25" s="6" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>نتائج</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>عدد الوظائف للسعوديين (لكل سنة)</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>البنك / أروقة</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr"/>
-      <c r="I26" s="6" t="inlineStr"/>
-      <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr"/>
-      <c r="L26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>أثر</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>إجمالي إيرادات الشركات المتخرجة</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>⚠ غير مُراجَع</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>البنك / أروقة</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr"/>
-      <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr"/>
-      <c r="I27" s="6" t="inlineStr"/>
-      <c r="J27" s="6" t="inlineStr"/>
-      <c r="K27" s="6" t="inlineStr"/>
-      <c r="L27" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5136,7 +5036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5319,7 +5219,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>جاهزية منصة التقييم RCAT وأدوات التأهيل</t>
+          <t>عدد الشراكات الفعّالة (المركز الوطني والوحدات الإشرافية)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -5334,7 +5234,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ركين</t>
+          <t>البنك / ركين</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
@@ -5345,12 +5245,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>مدخلات</t>
+          <t>أنشطة</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>عدد الشراكات الفعّالة (المركز الوطني والوحدات الإشرافية)</t>
+          <t>عدد الجمعيات التي خضعت لتقييم الجاهزية</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -5365,7 +5265,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>البنك / ركين</t>
+          <t>ركين</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr"/>
@@ -5381,7 +5281,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>عدد الجمعيات التي خضعت لتقييم الجاهزية</t>
+          <t>عدد ورش العمل الحضورية المنفّذة</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -5412,7 +5312,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>عدد ورش العمل الحضورية المنفّذة</t>
+          <t>عدد منسوبي الجمعيات المشاركين في الورش</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -5443,7 +5343,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>عدد منسوبي الجمعيات المشاركين في الورش</t>
+          <t>رضا المشاركين عن ورش العمل (%)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -5458,7 +5358,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>ركين</t>
+          <t>ركين (استبيان)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -5474,7 +5374,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>رضا المشاركين عن ورش العمل (%)</t>
+          <t>عدد اللقاءات المعرفية المنفّذة</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5489,7 +5389,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>ركين (استبيان)</t>
+          <t>ركين</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr"/>
@@ -5505,7 +5405,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>عدد اللقاءات المعرفية المنفّذة</t>
+          <t>عدد الزيارات الميدانية والجلسات الاستشارية المنفّذة</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -5531,12 +5431,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>أنشطة</t>
+          <t>مخرجات</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>عدد الزيارات الميدانية والجلسات الاستشارية المنفّذة</t>
+          <t>عدد الجمعيات المؤهَّلة — مسار تمكين (2026)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -5567,7 +5467,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>عدد الجمعيات المؤهَّلة — مسار تمكين (2026)</t>
+          <t>عدد الجمعيات المؤهَّلة — مسار تعظيم أثر (2026)</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -5598,7 +5498,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>عدد الجمعيات المؤهَّلة — مسار تعظيم أثر (2026)</t>
+          <t>عدد تقارير تقييم الجاهزية الصادرة</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -5629,7 +5529,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>عدد تقارير تقييم الجاهزية الصادرة</t>
+          <t>عدد خطط تفعيل المنافسات الحكومية المُعدّة</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -5655,12 +5555,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>مخرجات</t>
+          <t>نتائج</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>عدد خطط تفعيل المنافسات الحكومية المُعدّة</t>
+          <t>درجة جاهزية الإسناد (RCAT دخول/خروج)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -5686,12 +5586,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>نتائج</t>
+          <t>أثر</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>درجة جاهزية الإسناد (RCAT دخول/خروج)</t>
+          <t>عدد الجمعيات التي تقدّمت على فرص إسناد حكومية</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -5701,7 +5601,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>متوفر الآن ✓</t>
+          <t>يحتاج جلب</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -5722,7 +5622,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>عدد الجمعيات التي تقدّمت على فرص إسناد حكومية</t>
+          <t>عدد الجمعيات التي فازت بعقود إسناد حكومية</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -5745,37 +5645,6 @@
       <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>أثر</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>عدد الجمعيات التي فازت بعقود إسناد حكومية</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>يحتاج جلب</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>ركين</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr"/>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
content: apply ن4 reconciliation (p1 caveat, +p2_i05 rent, p3 +i27/-i16, p7 rebuild)
- p1_i16: append caveat «يُجمع من سجلات الجمعيات المنفّذة عند توفّرها»
- p2_i05: ADD متوسط الإيجار الشهري قبل البرنامج (نتائج, matrix)
- p3: ADD p3_i27 (ministry community-satisfaction record), REMOVE p3_i16 (flipped to استبيان)
- p7: rebuild from ن4 — 17 سجلات items, drop p7_i09 استبيان, re-id spend i19→i02
- regenerate al-ahli-sijillat-template.xlsx

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/al-ahli-sijillat-template.xlsx
+++ b/al-ahli-sijillat-template.xlsx
@@ -1333,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1713,22 +1713,22 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>قائمة الأسر المستفيدة (اسم + جوال + مدينة + عدد أفراد الأسرة)</t>
+          <t>متوسط الإيجار الشهري قبل البرنامج (لكل سنة)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>قائمة مستفيدين (PII)</t>
+          <t>مصفوفة سنوات</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>يحتاج إذن / إحالة</t>
+          <t>يحتاج جلب</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>الوزارة → (بإذن) البنك</t>
+          <t>الوزارة → البنك / المستفيد</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr"/>
@@ -1738,6 +1738,40 @@
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="6" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>نتائج</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>قائمة الأسر المستفيدة (اسم + جوال + مدينة + عدد أفراد الأسرة)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>قائمة مستفيدين (PII)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>يحتاج إذن / إحالة</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>الوزارة → (بإذن) البنك</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2800,7 +2834,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>تقييم الشركاء لأثر البرنامج البيئي</t>
+          <t>تقييم الوزارة/الشركاء لرضا المجتمع عن المبادرات البيئية (%)</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -5219,12 +5253,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>عدد الشراكات الفعّالة (المركز الوطني والوحدات الإشرافية)</t>
+          <t>جاهزية منصة التقييم RCAT وأدوات التأهيل</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>مصفوفة سنوات</t>
+          <t>وثيقة مرفقة</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -5234,7 +5268,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>البنك / ركين</t>
+          <t>ركين</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
@@ -5245,12 +5279,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>أنشطة</t>
+          <t>مدخلات</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>عدد الجمعيات التي خضعت لتقييم الجاهزية</t>
+          <t>عدد الشراكات الفعّالة (المركز الوطني والوحدات الإشرافية)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -5265,7 +5299,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>ركين</t>
+          <t>البنك / ركين</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr"/>
@@ -5281,7 +5315,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>عدد ورش العمل الحضورية المنفّذة</t>
+          <t>عدد الجمعيات التي خضعت لتقييم الجاهزية</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -5312,7 +5346,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>عدد منسوبي الجمعيات المشاركين في الورش</t>
+          <t>عدد ورش العمل الحضورية المنفّذة</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -5343,7 +5377,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>رضا المشاركين عن ورش العمل (%)</t>
+          <t>عدد منسوبي الجمعيات المشاركين في الورش</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -5358,7 +5392,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>ركين (استبيان)</t>
+          <t>ركين</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -5560,7 +5594,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>درجة جاهزية الإسناد (RCAT دخول/خروج)</t>
+          <t>درجة جاهزية الإسناد (تقييم RCAT دخول/خروج)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat(form): per-question add-year columns + رضا المستفيدات as held-record doc
- Matrix questions get a «+ أضف سنة» control; client appends extra year
  columns per question (editable 4-digit label, removable via × on added
  columns only). Added years + values persist in localStorage and restore
  on reload; empty added columns still persist.
- Excel export now uses the union of program base years + all client-added
  years across questions (sorted asc), RTL + Arabic headers preserved.
- رضا المستفيدات عن التدريب (p1_i13): matrix → document held-record shape,
  relabeled so it is clearly the client's existing questionnaire results
  handed over, not a new survey.
- Confirmed نسبة المتاجر النشطة and نسبة الفئات الأولى (100%) absent.
- Regenerated al-ahli-sijillat-template.xlsx from data.js.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/al-ahli-sijillat-template.xlsx
+++ b/al-ahli-sijillat-template.xlsx
@@ -956,12 +956,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>رضا المستفيدات عن التدريب (النتيجة سنوياً)</t>
+          <t>نتائج استبيان رضا المستفيدات عن التدريب (السجل لدى العميل)</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>مصفوفة سنوات</t>
+          <t>وثيقة مرفقة</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
content: remove carbon-footprint item p3_i19 from Program 3
Owner ruling: carbon-footprint (الفوت برنت / نسبة الخفض الكربوني) stays
off the client form — the firm pulls it from the ministry directly.
Also scrubbed the now-stale footprint sentence from the P3 note.
Regenerated al-ahli-sijillat-template.xlsx. Program 3: 21 -> 20 items.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/al-ahli-sijillat-template.xlsx
+++ b/al-ahli-sijillat-template.xlsx
@@ -1784,7 +1784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1796,13 +1796,9 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1822,7 +1818,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>السنوات مفترَضة 2022–2025 (يُؤكَّد). المساجد لا كونتاكت لها؛ الشركاء = وزارة البيئة. الفوت برنت يبدأ من السنة القادمة.</t>
+          <t>السنوات مفترَضة 2022–2025 (يُؤكَّد). المساجد لا كونتاكت لها؛ الشركاء = وزارة البيئة.</t>
         </is>
       </c>
     </row>
@@ -1874,35 +1870,15 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>حالة المستند/القائمة</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>العدد</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>2029</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t>حالة المستند/القائمة</t>
-        </is>
-      </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>العدد</t>
-        </is>
-      </c>
-      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>ملاحظات</t>
         </is>
@@ -1938,29 +1914,9 @@
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr"/>
-      <c r="O6" s="6" t="inlineStr"/>
-      <c r="P6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
+      <c r="L6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1992,29 +1948,9 @@
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2046,29 +1982,9 @@
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N8" s="6" t="inlineStr"/>
-      <c r="O8" s="6" t="inlineStr"/>
-      <c r="P8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2100,29 +2016,9 @@
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr"/>
-      <c r="P9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2154,29 +2050,9 @@
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M10" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N10" s="6" t="inlineStr"/>
-      <c r="O10" s="6" t="inlineStr"/>
-      <c r="P10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2208,29 +2084,9 @@
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr"/>
-      <c r="O11" s="6" t="inlineStr"/>
-      <c r="P11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2262,29 +2118,9 @@
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N12" s="6" t="inlineStr"/>
-      <c r="O12" s="6" t="inlineStr"/>
-      <c r="P12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2316,29 +2152,9 @@
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N13" s="6" t="inlineStr"/>
-      <c r="O13" s="6" t="inlineStr"/>
-      <c r="P13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2370,29 +2186,9 @@
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N14" s="6" t="inlineStr"/>
-      <c r="O14" s="6" t="inlineStr"/>
-      <c r="P14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
+      <c r="L14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2424,29 +2220,9 @@
       <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N15" s="6" t="inlineStr"/>
-      <c r="O15" s="6" t="inlineStr"/>
-      <c r="P15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2478,29 +2254,9 @@
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr"/>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M16" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N16" s="6" t="inlineStr"/>
-      <c r="O16" s="6" t="inlineStr"/>
-      <c r="P16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2532,29 +2288,9 @@
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2586,29 +2322,9 @@
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M18" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N18" s="6" t="inlineStr"/>
-      <c r="O18" s="6" t="inlineStr"/>
-      <c r="P18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2640,29 +2356,9 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N19" s="6" t="inlineStr"/>
-      <c r="O19" s="6" t="inlineStr"/>
-      <c r="P19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2694,29 +2390,9 @@
       <c r="G20" s="6" t="inlineStr"/>
       <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N20" s="6" t="inlineStr"/>
-      <c r="O20" s="6" t="inlineStr"/>
-      <c r="P20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2748,29 +2424,9 @@
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2802,29 +2458,9 @@
       <c r="G22" s="6" t="inlineStr"/>
       <c r="H22" s="6" t="inlineStr"/>
       <c r="I22" s="6" t="inlineStr"/>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N22" s="6" t="inlineStr"/>
-      <c r="O22" s="6" t="inlineStr"/>
-      <c r="P22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
+      <c r="L22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2859,10 +2495,6 @@
       <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr"/>
-      <c r="M23" s="6" t="inlineStr"/>
-      <c r="N23" s="6" t="inlineStr"/>
-      <c r="O23" s="6" t="inlineStr"/>
-      <c r="P23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2894,29 +2526,9 @@
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr"/>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N24" s="6" t="inlineStr"/>
-      <c r="O24" s="6" t="inlineStr"/>
-      <c r="P24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2948,83 +2560,9 @@
       <c r="G25" s="6" t="inlineStr"/>
       <c r="H25" s="6" t="inlineStr"/>
       <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N25" s="6" t="inlineStr"/>
-      <c r="O25" s="6" t="inlineStr"/>
-      <c r="P25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>أثر</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>الفوت برنت / نسبة الخفض الكربوني (مانجروف وغيره)</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>مصفوفة سنوات</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>يحتاج جلب</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>البنك / الوزارة</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr"/>
-      <c r="K26" s="6" t="inlineStr"/>
-      <c r="L26" s="6" t="inlineStr"/>
-      <c r="M26" s="6" t="inlineStr"/>
-      <c r="N26" s="6" t="inlineStr"/>
-      <c r="O26" s="6" t="inlineStr"/>
-      <c r="P26" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>